<commit_message>
new cartographie & correspondance
</commit_message>
<xml_diff>
--- a/Cartographie Audit IT [PERSONAL]/Cartographie_Risques_IT_Complete.xlsx
+++ b/Cartographie Audit IT [PERSONAL]/Cartographie_Risques_IT_Complete.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eleve04\Documents\Github\ProjetGithub\PROJECTS_NDOUDI_Nimrod\Cartographie Audit IT [PERSONAL]\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5789F9DB-F4A5-4F45-B425-BCAB24E4CE3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5E625D-0B40-40E8-9A0B-418928F92ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CARTOGRAPHIE" sheetId="1" r:id="rId1"/>
@@ -992,17 +992,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1034,6 +1025,15 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1365,22 +1365,22 @@
       <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="G1" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="28" t="s">
+      <c r="J1" s="25" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -1388,34 +1388,34 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="F2" s="17" t="s">
+      <c r="F2" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="H2" s="25">
+      <c r="H2" s="22">
         <v>2</v>
       </c>
-      <c r="I2" s="25">
+      <c r="I2" s="22">
         <v>5</v>
       </c>
-      <c r="J2" s="29">
+      <c r="J2" s="26">
         <v>10</v>
       </c>
       <c r="K2" s="4" t="s">
@@ -1423,32 +1423,32 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="30"/>
+      <c r="B3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="H3" s="26">
-        <v>3</v>
-      </c>
-      <c r="I3" s="26">
+      <c r="H3" s="23">
+        <v>3</v>
+      </c>
+      <c r="I3" s="23">
         <v>4</v>
       </c>
-      <c r="J3" s="30">
+      <c r="J3" s="27">
         <v>12</v>
       </c>
       <c r="K3" s="2" t="s">
@@ -1456,32 +1456,32 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="30"/>
+      <c r="B4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="H4" s="26">
-        <v>3</v>
-      </c>
-      <c r="I4" s="26">
+      <c r="H4" s="23">
+        <v>3</v>
+      </c>
+      <c r="I4" s="23">
         <v>4</v>
       </c>
-      <c r="J4" s="30">
+      <c r="J4" s="27">
         <v>12</v>
       </c>
       <c r="K4" s="2" t="s">
@@ -1489,32 +1489,32 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11" t="s">
+      <c r="A5" s="31"/>
+      <c r="B5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="20" t="s">
         <v>200</v>
       </c>
-      <c r="H5" s="27">
-        <v>3</v>
-      </c>
-      <c r="I5" s="27">
+      <c r="H5" s="24">
+        <v>3</v>
+      </c>
+      <c r="I5" s="24">
         <v>4</v>
       </c>
-      <c r="J5" s="31">
+      <c r="J5" s="28">
         <v>12</v>
       </c>
       <c r="K5" s="3" t="s">
@@ -1522,34 +1522,34 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="H6" s="25">
-        <v>3</v>
-      </c>
-      <c r="I6" s="25">
+      <c r="H6" s="22">
+        <v>3</v>
+      </c>
+      <c r="I6" s="22">
         <v>4</v>
       </c>
-      <c r="J6" s="29">
+      <c r="J6" s="26">
         <v>12</v>
       </c>
       <c r="K6" s="4" t="s">
@@ -1557,32 +1557,32 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="8"/>
-      <c r="B7" s="9" t="s">
+      <c r="A7" s="30"/>
+      <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="H7" s="26">
+      <c r="H7" s="23">
         <v>4</v>
       </c>
-      <c r="I7" s="26">
+      <c r="I7" s="23">
         <v>5</v>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="27">
         <v>20</v>
       </c>
       <c r="K7" s="2" t="s">
@@ -1590,32 +1590,32 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9" t="s">
+      <c r="A8" s="30"/>
+      <c r="B8" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="H8" s="26">
-        <v>3</v>
-      </c>
-      <c r="I8" s="26">
+      <c r="H8" s="23">
+        <v>3</v>
+      </c>
+      <c r="I8" s="23">
         <v>5</v>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="27">
         <v>15</v>
       </c>
       <c r="K8" s="2" t="s">
@@ -1623,32 +1623,32 @@
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11" t="s">
+      <c r="A9" s="31"/>
+      <c r="B9" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="H9" s="27">
-        <v>3</v>
-      </c>
-      <c r="I9" s="27">
+      <c r="H9" s="24">
+        <v>3</v>
+      </c>
+      <c r="I9" s="24">
         <v>4</v>
       </c>
-      <c r="J9" s="31">
+      <c r="J9" s="28">
         <v>12</v>
       </c>
       <c r="K9" s="3" t="s">
@@ -1656,34 +1656,34 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="G10" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="H10" s="25">
-        <v>3</v>
-      </c>
-      <c r="I10" s="25">
+      <c r="H10" s="22">
+        <v>3</v>
+      </c>
+      <c r="I10" s="22">
         <v>5</v>
       </c>
-      <c r="J10" s="29">
+      <c r="J10" s="26">
         <v>15</v>
       </c>
       <c r="K10" s="4" t="s">
@@ -1691,32 +1691,32 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="30"/>
+      <c r="B11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="9" t="s">
+      <c r="D11" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="H11" s="26">
-        <v>3</v>
-      </c>
-      <c r="I11" s="26">
+      <c r="H11" s="23">
+        <v>3</v>
+      </c>
+      <c r="I11" s="23">
         <v>4</v>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="27">
         <v>12</v>
       </c>
       <c r="K11" s="2" t="s">
@@ -1724,32 +1724,32 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="30"/>
+      <c r="B12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="G12" s="22" t="s">
+      <c r="G12" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="H12" s="26">
+      <c r="H12" s="23">
         <v>2</v>
       </c>
-      <c r="I12" s="26">
+      <c r="I12" s="23">
         <v>4</v>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="27">
         <v>8</v>
       </c>
       <c r="K12" s="2" t="s">
@@ -1757,32 +1757,32 @@
       </c>
     </row>
     <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11" t="s">
+      <c r="A13" s="31"/>
+      <c r="B13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="20" t="s">
         <v>208</v>
       </c>
-      <c r="H13" s="27">
-        <v>3</v>
-      </c>
-      <c r="I13" s="27">
+      <c r="H13" s="24">
+        <v>3</v>
+      </c>
+      <c r="I13" s="24">
         <v>5</v>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="28">
         <v>15</v>
       </c>
       <c r="K13" s="3" t="s">
@@ -1790,34 +1790,34 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="G14" s="21" t="s">
+      <c r="G14" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="H14" s="25">
-        <v>3</v>
-      </c>
-      <c r="I14" s="25">
+      <c r="H14" s="22">
+        <v>3</v>
+      </c>
+      <c r="I14" s="22">
         <v>4</v>
       </c>
-      <c r="J14" s="29">
+      <c r="J14" s="26">
         <v>12</v>
       </c>
       <c r="K14" s="4" t="s">
@@ -1825,32 +1825,32 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="30"/>
+      <c r="B15" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="D15" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="F15" s="18" t="s">
+      <c r="F15" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="G15" s="22" t="s">
+      <c r="G15" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="H15" s="26">
-        <v>3</v>
-      </c>
-      <c r="I15" s="26">
+      <c r="H15" s="23">
+        <v>3</v>
+      </c>
+      <c r="I15" s="23">
         <v>5</v>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="27">
         <v>15</v>
       </c>
       <c r="K15" s="2" t="s">
@@ -1858,32 +1858,32 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="30"/>
+      <c r="B16" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="E16" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="F16" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="H16" s="26">
-        <v>3</v>
-      </c>
-      <c r="I16" s="26">
+      <c r="H16" s="23">
+        <v>3</v>
+      </c>
+      <c r="I16" s="23">
         <v>4</v>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="27">
         <v>12</v>
       </c>
       <c r="K16" s="2" t="s">
@@ -1891,32 +1891,32 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11" t="s">
+      <c r="A17" s="31"/>
+      <c r="B17" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="24">
         <v>4</v>
       </c>
-      <c r="I17" s="27">
+      <c r="I17" s="24">
         <v>4</v>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="28">
         <v>16</v>
       </c>
       <c r="K17" s="3" t="s">
@@ -1924,34 +1924,34 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="G18" s="21" t="s">
+      <c r="G18" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="22">
         <v>4</v>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="22">
         <v>4</v>
       </c>
-      <c r="J18" s="29">
+      <c r="J18" s="26">
         <v>16</v>
       </c>
       <c r="K18" s="4" t="s">
@@ -1959,32 +1959,32 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="8"/>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="30"/>
+      <c r="B19" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="9" t="s">
+      <c r="D19" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="E19" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="H19" s="26">
-        <v>3</v>
-      </c>
-      <c r="I19" s="26">
+      <c r="H19" s="23">
+        <v>3</v>
+      </c>
+      <c r="I19" s="23">
         <v>5</v>
       </c>
-      <c r="J19" s="30">
+      <c r="J19" s="27">
         <v>15</v>
       </c>
       <c r="K19" s="2" t="s">
@@ -1992,32 +1992,32 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="8"/>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="30"/>
+      <c r="B20" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D20" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="E20" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="G20" s="22" t="s">
+      <c r="G20" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="H20" s="26">
-        <v>3</v>
-      </c>
-      <c r="I20" s="26">
+      <c r="H20" s="23">
+        <v>3</v>
+      </c>
+      <c r="I20" s="23">
         <v>5</v>
       </c>
-      <c r="J20" s="30">
+      <c r="J20" s="27">
         <v>15</v>
       </c>
       <c r="K20" s="2" t="s">
@@ -2025,32 +2025,32 @@
       </c>
     </row>
     <row r="21" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11" t="s">
+      <c r="A21" s="31"/>
+      <c r="B21" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="F21" s="19" t="s">
+      <c r="F21" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G21" s="20" t="s">
         <v>210</v>
       </c>
-      <c r="H21" s="27">
-        <v>3</v>
-      </c>
-      <c r="I21" s="27">
+      <c r="H21" s="24">
+        <v>3</v>
+      </c>
+      <c r="I21" s="24">
         <v>4</v>
       </c>
-      <c r="J21" s="31">
+      <c r="J21" s="28">
         <v>12</v>
       </c>
       <c r="K21" s="3" t="s">
@@ -2058,34 +2058,34 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E22" s="13" t="s">
+      <c r="E22" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G22" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="H22" s="25">
-        <v>3</v>
-      </c>
-      <c r="I22" s="25">
+      <c r="H22" s="22">
+        <v>3</v>
+      </c>
+      <c r="I22" s="22">
         <v>5</v>
       </c>
-      <c r="J22" s="29">
+      <c r="J22" s="26">
         <v>15</v>
       </c>
       <c r="K22" s="4" t="s">
@@ -2093,32 +2093,32 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="9" t="s">
+      <c r="A23" s="30"/>
+      <c r="B23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="E23" s="14" t="s">
+      <c r="E23" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="G23" s="22" t="s">
+      <c r="G23" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="H23" s="26">
+      <c r="H23" s="23">
         <v>4</v>
       </c>
-      <c r="I23" s="26">
+      <c r="I23" s="23">
         <v>4</v>
       </c>
-      <c r="J23" s="30">
+      <c r="J23" s="27">
         <v>16</v>
       </c>
       <c r="K23" s="2" t="s">
@@ -2126,32 +2126,32 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="9" t="s">
+      <c r="A24" s="30"/>
+      <c r="B24" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="E24" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="G24" s="22" t="s">
+      <c r="G24" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="H24" s="26">
-        <v>3</v>
-      </c>
-      <c r="I24" s="26">
+      <c r="H24" s="23">
+        <v>3</v>
+      </c>
+      <c r="I24" s="23">
         <v>4</v>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="27">
         <v>12</v>
       </c>
       <c r="K24" s="2" t="s">
@@ -2159,32 +2159,32 @@
       </c>
     </row>
     <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="11" t="s">
+      <c r="A25" s="31"/>
+      <c r="B25" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="11" t="s">
+      <c r="C25" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="D25" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="E25" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="F25" s="19" t="s">
+      <c r="F25" s="16" t="s">
         <v>186</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" s="20" t="s">
         <v>205</v>
       </c>
-      <c r="H25" s="27">
+      <c r="H25" s="24">
         <v>4</v>
       </c>
-      <c r="I25" s="27">
+      <c r="I25" s="24">
         <v>4</v>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="28">
         <v>16</v>
       </c>
       <c r="K25" s="3" t="s">
@@ -2192,34 +2192,34 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="E26" s="13" t="s">
+      <c r="E26" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="G26" s="21" t="s">
+      <c r="G26" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="H26" s="25">
-        <v>3</v>
-      </c>
-      <c r="I26" s="25">
+      <c r="H26" s="22">
+        <v>3</v>
+      </c>
+      <c r="I26" s="22">
         <v>5</v>
       </c>
-      <c r="J26" s="29">
+      <c r="J26" s="26">
         <v>15</v>
       </c>
       <c r="K26" s="4" t="s">
@@ -2227,32 +2227,32 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="9" t="s">
+      <c r="A27" s="30"/>
+      <c r="B27" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="D27" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="E27" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="F27" s="18" t="s">
+      <c r="F27" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="G27" s="22" t="s">
+      <c r="G27" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="H27" s="26">
-        <v>3</v>
-      </c>
-      <c r="I27" s="26">
+      <c r="H27" s="23">
+        <v>3</v>
+      </c>
+      <c r="I27" s="23">
         <v>5</v>
       </c>
-      <c r="J27" s="30">
+      <c r="J27" s="27">
         <v>15</v>
       </c>
       <c r="K27" s="2" t="s">
@@ -2260,32 +2260,32 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="9" t="s">
+      <c r="A28" s="30"/>
+      <c r="B28" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="F28" s="18" t="s">
+      <c r="F28" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="G28" s="22" t="s">
+      <c r="G28" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="H28" s="26">
-        <v>3</v>
-      </c>
-      <c r="I28" s="26">
+      <c r="H28" s="23">
+        <v>3</v>
+      </c>
+      <c r="I28" s="23">
         <v>4</v>
       </c>
-      <c r="J28" s="30">
+      <c r="J28" s="27">
         <v>12</v>
       </c>
       <c r="K28" s="2" t="s">
@@ -2293,32 +2293,32 @@
       </c>
     </row>
     <row r="29" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="10"/>
-      <c r="B29" s="11" t="s">
+      <c r="A29" s="31"/>
+      <c r="B29" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C29" s="11" t="s">
+      <c r="C29" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="F29" s="19" t="s">
+      <c r="F29" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="G29" s="23" t="s">
+      <c r="G29" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="H29" s="27">
-        <v>3</v>
-      </c>
-      <c r="I29" s="27">
+      <c r="H29" s="24">
+        <v>3</v>
+      </c>
+      <c r="I29" s="24">
         <v>5</v>
       </c>
-      <c r="J29" s="31">
+      <c r="J29" s="28">
         <v>15</v>
       </c>
       <c r="K29" s="3" t="s">
@@ -2326,34 +2326,34 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="F30" s="17" t="s">
+      <c r="F30" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="G30" s="21" t="s">
+      <c r="G30" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="H30" s="25">
+      <c r="H30" s="22">
         <v>2</v>
       </c>
-      <c r="I30" s="25">
+      <c r="I30" s="22">
         <v>5</v>
       </c>
-      <c r="J30" s="29">
+      <c r="J30" s="26">
         <v>10</v>
       </c>
       <c r="K30" s="4" t="s">
@@ -2361,32 +2361,32 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="8"/>
-      <c r="B31" s="9" t="s">
+      <c r="A31" s="30"/>
+      <c r="B31" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="E31" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="F31" s="18" t="s">
+      <c r="F31" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="G31" s="22" t="s">
+      <c r="G31" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="H31" s="26">
-        <v>3</v>
-      </c>
-      <c r="I31" s="26">
+      <c r="H31" s="23">
+        <v>3</v>
+      </c>
+      <c r="I31" s="23">
         <v>5</v>
       </c>
-      <c r="J31" s="30">
+      <c r="J31" s="27">
         <v>15</v>
       </c>
       <c r="K31" s="2" t="s">
@@ -2394,32 +2394,32 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="8"/>
-      <c r="B32" s="9" t="s">
+      <c r="A32" s="30"/>
+      <c r="B32" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="D32" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="E32" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="F32" s="18" t="s">
+      <c r="F32" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="G32" s="22" t="s">
+      <c r="G32" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="H32" s="26">
-        <v>3</v>
-      </c>
-      <c r="I32" s="26">
+      <c r="H32" s="23">
+        <v>3</v>
+      </c>
+      <c r="I32" s="23">
         <v>4</v>
       </c>
-      <c r="J32" s="30">
+      <c r="J32" s="27">
         <v>12</v>
       </c>
       <c r="K32" s="2" t="s">
@@ -2427,32 +2427,32 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11" t="s">
+      <c r="A33" s="31"/>
+      <c r="B33" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="11" t="s">
+      <c r="C33" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="8" t="s">
         <v>132</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="E33" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="F33" s="19" t="s">
+      <c r="F33" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="G33" s="23" t="s">
+      <c r="G33" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="H33" s="27">
-        <v>3</v>
-      </c>
-      <c r="I33" s="27">
+      <c r="H33" s="24">
+        <v>3</v>
+      </c>
+      <c r="I33" s="24">
         <v>4</v>
       </c>
-      <c r="J33" s="31">
+      <c r="J33" s="28">
         <v>12</v>
       </c>
       <c r="K33" s="3" t="s">
@@ -2460,34 +2460,34 @@
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="10" t="s">
         <v>164</v>
       </c>
-      <c r="F34" s="17" t="s">
+      <c r="F34" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="G34" s="21" t="s">
+      <c r="G34" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="H34" s="25">
-        <v>3</v>
-      </c>
-      <c r="I34" s="25">
+      <c r="H34" s="22">
+        <v>3</v>
+      </c>
+      <c r="I34" s="22">
         <v>5</v>
       </c>
-      <c r="J34" s="29">
+      <c r="J34" s="26">
         <v>15</v>
       </c>
       <c r="K34" s="4" t="s">
@@ -2495,32 +2495,32 @@
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="8"/>
-      <c r="B35" s="9" t="s">
+      <c r="A35" s="30"/>
+      <c r="B35" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="E35" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="F35" s="18" t="s">
+      <c r="F35" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="G35" s="22" t="s">
+      <c r="G35" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="H35" s="26">
-        <v>3</v>
-      </c>
-      <c r="I35" s="26">
+      <c r="H35" s="23">
+        <v>3</v>
+      </c>
+      <c r="I35" s="23">
         <v>5</v>
       </c>
-      <c r="J35" s="30">
+      <c r="J35" s="27">
         <v>15</v>
       </c>
       <c r="K35" s="2" t="s">
@@ -2528,32 +2528,32 @@
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="8"/>
-      <c r="B36" s="9" t="s">
+      <c r="A36" s="30"/>
+      <c r="B36" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="E36" s="14" t="s">
+      <c r="E36" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="F36" s="18" t="s">
+      <c r="F36" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="G36" s="22" t="s">
+      <c r="G36" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="H36" s="26">
+      <c r="H36" s="23">
         <v>2</v>
       </c>
-      <c r="I36" s="26">
+      <c r="I36" s="23">
         <v>5</v>
       </c>
-      <c r="J36" s="30">
+      <c r="J36" s="27">
         <v>10</v>
       </c>
       <c r="K36" s="2" t="s">
@@ -2561,32 +2561,32 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11" t="s">
+      <c r="A37" s="31"/>
+      <c r="B37" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E37" s="15" t="s">
+      <c r="E37" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="F37" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="G37" s="23" t="s">
+      <c r="G37" s="20" t="s">
         <v>217</v>
       </c>
-      <c r="H37" s="27">
-        <v>3</v>
-      </c>
-      <c r="I37" s="27">
+      <c r="H37" s="24">
+        <v>3</v>
+      </c>
+      <c r="I37" s="24">
         <v>4</v>
       </c>
-      <c r="J37" s="31">
+      <c r="J37" s="28">
         <v>12</v>
       </c>
       <c r="K37" s="3" t="s">
@@ -2594,34 +2594,34 @@
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="B38" s="7" t="s">
+      <c r="B38" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E38" s="13" t="s">
+      <c r="E38" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="F38" s="17" t="s">
+      <c r="F38" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="G38" s="21" t="s">
+      <c r="G38" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="H38" s="25">
-        <v>3</v>
-      </c>
-      <c r="I38" s="25">
+      <c r="H38" s="22">
+        <v>3</v>
+      </c>
+      <c r="I38" s="22">
         <v>4</v>
       </c>
-      <c r="J38" s="29">
+      <c r="J38" s="26">
         <v>12</v>
       </c>
       <c r="K38" s="4" t="s">
@@ -2629,32 +2629,32 @@
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="8"/>
-      <c r="B39" s="9" t="s">
+      <c r="A39" s="30"/>
+      <c r="B39" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="D39" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="E39" s="14" t="s">
+      <c r="E39" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="F39" s="18" t="s">
+      <c r="F39" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="G39" s="22" t="s">
+      <c r="G39" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="H39" s="26">
-        <v>3</v>
-      </c>
-      <c r="I39" s="26">
+      <c r="H39" s="23">
+        <v>3</v>
+      </c>
+      <c r="I39" s="23">
         <v>5</v>
       </c>
-      <c r="J39" s="30">
+      <c r="J39" s="27">
         <v>15</v>
       </c>
       <c r="K39" s="2" t="s">
@@ -2662,32 +2662,32 @@
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="8"/>
-      <c r="B40" s="9" t="s">
+      <c r="A40" s="30"/>
+      <c r="B40" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="E40" s="14" t="s">
+      <c r="E40" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="F40" s="18" t="s">
+      <c r="F40" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="G40" s="22" t="s">
+      <c r="G40" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="H40" s="26">
-        <v>3</v>
-      </c>
-      <c r="I40" s="26">
+      <c r="H40" s="23">
+        <v>3</v>
+      </c>
+      <c r="I40" s="23">
         <v>5</v>
       </c>
-      <c r="J40" s="30">
+      <c r="J40" s="27">
         <v>15</v>
       </c>
       <c r="K40" s="2" t="s">
@@ -2695,32 +2695,32 @@
       </c>
     </row>
     <row r="41" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="10"/>
-      <c r="B41" s="11" t="s">
+      <c r="A41" s="31"/>
+      <c r="B41" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="C41" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="11" t="s">
+      <c r="D41" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="E41" s="15" t="s">
+      <c r="E41" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="F41" s="19" t="s">
+      <c r="F41" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="G41" s="23" t="s">
+      <c r="G41" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="H41" s="27">
-        <v>3</v>
-      </c>
-      <c r="I41" s="27">
+      <c r="H41" s="24">
+        <v>3</v>
+      </c>
+      <c r="I41" s="24">
         <v>4</v>
       </c>
-      <c r="J41" s="31">
+      <c r="J41" s="28">
         <v>12</v>
       </c>
       <c r="K41" s="3" t="s">

</xml_diff>